<commit_message>
ISP címzés excelben elkészítve
</commit_message>
<xml_diff>
--- a/Network/cimzes.xlsx
+++ b/Network/cimzes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github Repo\final-project-2025-26\Network\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A749ECDE-4091-4F7C-ABBF-57E308866B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732AA075-24A0-4FE7-9A86-15BF42C83C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="15" windowWidth="14400" windowHeight="15600" activeTab="2" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6F35F872-ABCC-42C2-B031-C1DE53122CDE}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="186">
   <si>
     <t>Név</t>
   </si>
@@ -337,6 +337,255 @@
   </si>
   <si>
     <t>Gig6/0</t>
+  </si>
+  <si>
+    <t>172.16.0.4/30</t>
+  </si>
+  <si>
+    <t>172.16.0.8/30</t>
+  </si>
+  <si>
+    <t>172.16.0.12/30</t>
+  </si>
+  <si>
+    <t>172.16.0.16/30</t>
+  </si>
+  <si>
+    <t>172.16.0.20/30</t>
+  </si>
+  <si>
+    <t>172.16.0.24/30</t>
+  </si>
+  <si>
+    <t>172.16.0.28/30</t>
+  </si>
+  <si>
+    <t>172.16.0.32/30</t>
+  </si>
+  <si>
+    <t>172.16.0.36/30</t>
+  </si>
+  <si>
+    <t>172.16.0.40/30</t>
+  </si>
+  <si>
+    <t>172.16.0.44/30</t>
+  </si>
+  <si>
+    <t>172.16.0.48/30</t>
+  </si>
+  <si>
+    <t>172.16.0.52/30</t>
+  </si>
+  <si>
+    <t>172.16.0.56/30</t>
+  </si>
+  <si>
+    <t>172.16.0.60/30</t>
+  </si>
+  <si>
+    <t>172.16.0.64/30</t>
+  </si>
+  <si>
+    <t>172.16.0.68/30</t>
+  </si>
+  <si>
+    <t>172.16.0.72/30</t>
+  </si>
+  <si>
+    <t>172.16.0.76/30</t>
+  </si>
+  <si>
+    <t>172.16.0.80/30</t>
+  </si>
+  <si>
+    <t>172.16.0.84/30</t>
+  </si>
+  <si>
+    <t>172.16.0.88/30</t>
+  </si>
+  <si>
+    <t>172.16.0.92/30</t>
+  </si>
+  <si>
+    <t>172.16.0.96/30</t>
+  </si>
+  <si>
+    <t>172.16.0.100/30</t>
+  </si>
+  <si>
+    <t>172.16.0.104/30</t>
+  </si>
+  <si>
+    <t>172.16.0.108/30</t>
+  </si>
+  <si>
+    <t>172.16.0.1</t>
+  </si>
+  <si>
+    <t>172.16.0.2</t>
+  </si>
+  <si>
+    <t>172.16.0.5</t>
+  </si>
+  <si>
+    <t>172.16.0.6</t>
+  </si>
+  <si>
+    <t>172.16.0.9</t>
+  </si>
+  <si>
+    <t>172.16.0.13</t>
+  </si>
+  <si>
+    <t>172.16.0.17</t>
+  </si>
+  <si>
+    <t>172.16.0.21</t>
+  </si>
+  <si>
+    <t>172.16.0.25</t>
+  </si>
+  <si>
+    <t>172.16.0.10</t>
+  </si>
+  <si>
+    <t>172.16.0.14</t>
+  </si>
+  <si>
+    <t>172.16.0.18</t>
+  </si>
+  <si>
+    <t>172.16.0.22</t>
+  </si>
+  <si>
+    <t>172.16.0.26</t>
+  </si>
+  <si>
+    <t>172.16.0.29</t>
+  </si>
+  <si>
+    <t>172.16.0.30</t>
+  </si>
+  <si>
+    <t>172.16.0.33</t>
+  </si>
+  <si>
+    <t>172.16.0.37</t>
+  </si>
+  <si>
+    <t>172.16.0.41</t>
+  </si>
+  <si>
+    <t>172.16.0.45</t>
+  </si>
+  <si>
+    <t>172.16.0.49</t>
+  </si>
+  <si>
+    <t>172.16.0.34</t>
+  </si>
+  <si>
+    <t>172.16.0.38</t>
+  </si>
+  <si>
+    <t>172.16.0.42</t>
+  </si>
+  <si>
+    <t>172.16.0.46</t>
+  </si>
+  <si>
+    <t>172.16.0.50</t>
+  </si>
+  <si>
+    <t>172.16.0.53</t>
+  </si>
+  <si>
+    <t>172.16.0.54</t>
+  </si>
+  <si>
+    <t>172.16.0.57</t>
+  </si>
+  <si>
+    <t>172.16.0.61</t>
+  </si>
+  <si>
+    <t>172.16.0.65</t>
+  </si>
+  <si>
+    <t>172.16.0.69</t>
+  </si>
+  <si>
+    <t>172.16.0.73</t>
+  </si>
+  <si>
+    <t>172.16.0.77</t>
+  </si>
+  <si>
+    <t>172.16.0.81</t>
+  </si>
+  <si>
+    <t>172.16.0.85</t>
+  </si>
+  <si>
+    <t>172.16.0.89</t>
+  </si>
+  <si>
+    <t>172.16.0.93</t>
+  </si>
+  <si>
+    <t>172.16.0.97</t>
+  </si>
+  <si>
+    <t>172.16.0.101</t>
+  </si>
+  <si>
+    <t>172.16.0.105</t>
+  </si>
+  <si>
+    <t>172.16.0.109</t>
+  </si>
+  <si>
+    <t>172.16.0.58</t>
+  </si>
+  <si>
+    <t>172.16.0.62</t>
+  </si>
+  <si>
+    <t>172.16.0.66</t>
+  </si>
+  <si>
+    <t>172.16.0.70</t>
+  </si>
+  <si>
+    <t>172.16.0.74</t>
+  </si>
+  <si>
+    <t>172.16.0.78</t>
+  </si>
+  <si>
+    <t>172.16.0.82</t>
+  </si>
+  <si>
+    <t>172.16.0.86</t>
+  </si>
+  <si>
+    <t>172.16.0.90</t>
+  </si>
+  <si>
+    <t>172.16.0.94</t>
+  </si>
+  <si>
+    <t>172.16.0.98</t>
+  </si>
+  <si>
+    <t>172.16.0.102</t>
+  </si>
+  <si>
+    <t>172.16.0.106</t>
+  </si>
+  <si>
+    <t>172.16.0.110</t>
   </si>
 </sst>
 </file>
@@ -452,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -486,6 +735,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -1088,472 +1338,833 @@
   <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+      <c r="A1" s="19"/>
+      <c r="B1" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="19" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="19" t="s">
         <v>95</v>
       </c>
+      <c r="D2" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="19" t="s">
         <v>88</v>
       </c>
+      <c r="B3" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="19" t="s">
         <v>89</v>
       </c>
+      <c r="B4" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="19" t="s">
         <v>90</v>
       </c>
+      <c r="B5" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="19" t="s">
         <v>91</v>
       </c>
+      <c r="B6" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="19" t="s">
         <v>92</v>
       </c>
+      <c r="B7" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="19" t="s">
         <v>93</v>
       </c>
+      <c r="B8" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" s="19" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="19" t="s">
         <v>94</v>
       </c>
+      <c r="B9" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C12" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D12" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="11" t="s">
         <v>96</v>
       </c>
+      <c r="F12" s="11" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D13" t="s">
+      <c r="C13" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="11" t="s">
         <v>96</v>
       </c>
+      <c r="F13" s="11" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D14" t="s">
+      <c r="C14" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="11" t="s">
         <v>96</v>
       </c>
+      <c r="F14" s="11" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D15" t="s">
+      <c r="C15" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="11" t="s">
         <v>96</v>
       </c>
+      <c r="F15" s="11" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D16" t="s">
+      <c r="C16" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="11" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="F16" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D17" t="s">
+      <c r="C17" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="11" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="F17" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D18" t="s">
+      <c r="C18" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="11" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="F18" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D19" t="s">
+      <c r="C19" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="F19" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D20" t="s">
+      <c r="C20" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="F20" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D21" t="s">
+      <c r="C21" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="F21" s="11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D22" t="s">
+      <c r="C22" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="F22" s="11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D23" t="s">
+      <c r="C23" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="F23" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D24" t="s">
+      <c r="C24" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="11" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="F24" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D25" t="s">
+      <c r="C25" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="F25" s="11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D26" t="s">
+      <c r="C26" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="F26" s="11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D27" t="s">
+      <c r="C27" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="F27" s="11" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D28" t="s">
+      <c r="C28" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="F28" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D29" t="s">
+      <c r="C29" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="F29" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D30" t="s">
+      <c r="C30" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="F30" s="11" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D31" t="s">
+      <c r="C31" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="F31" s="11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D32" t="s">
+      <c r="C32" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="F32" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D33" t="s">
+      <c r="C33" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D33" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="F33" s="11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D34" t="s">
+      <c r="C34" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="11" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="F34" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D35" t="s">
+      <c r="C35" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="11" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="F35" s="11" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D36" t="s">
+      <c r="C36" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D36" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="11" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="F36" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D37" t="s">
+      <c r="C37" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D37" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="F37" s="11" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D38" t="s">
+      <c r="C38" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D38" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="F38" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D39" t="s">
+      <c r="C39" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D39" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="11" t="s">
         <v>102</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>